<commit_message>
docs(examples): minor update to charts-line.xlsx
</commit_message>
<xml_diff>
--- a/examples/excel/charts-line.xlsx
+++ b/examples/excel/charts-line.xlsx
@@ -3,13 +3,13 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="Ref14dd27bc574f96"/>
-    <x:sheet name="2-Line Styles" sheetId="3" r:id="Rd3a552787c06462f"/>
-    <x:sheet name="3-Line Variants" sheetId="4" r:id="Rc5d441f08a9d4e05"/>
-    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="R14f48eba710c4b22"/>
-    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="Re081da5ad2174cfe"/>
-    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="R32bfe97758f3421a"/>
-    <x:sheet name="7-Line Elements" sheetId="8" r:id="R81fa9589da944736"/>
+    <x:sheet name="1-Line Fundamentals" sheetId="2" r:id="R07348e2e24d64303"/>
+    <x:sheet name="2-Line Styles" sheetId="3" r:id="Rabcd157a92f14e19"/>
+    <x:sheet name="3-Line Variants" sheetId="4" r:id="Rb3d2e0be611240a6"/>
+    <x:sheet name="4-Axis &amp; Gridlines" sheetId="5" r:id="R6b7b79b4bb164d73"/>
+    <x:sheet name="5-Labels &amp; Legend" sheetId="6" r:id="R56a36020a7474f56"/>
+    <x:sheet name="6-Effects &amp; Advanced" sheetId="7" r:id="R273f7a256bca4711"/>
+    <x:sheet name="7-Line Elements" sheetId="8" r:id="Ra8030ba92ed44110"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -862,7 +862,7 @@
     </c:view3D>
     <c:plotArea>
       <c:layout/>
-      <c:lineChart>
+      <c:line3DChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
@@ -1269,10 +1269,9 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:marker val="1"/>
         <c:axId val="1"/>
         <c:axId val="2"/>
-      </c:lineChart>
+      </c:line3DChart>
       <c:catAx>
         <c:axId val="1"/>
         <c:scaling>
@@ -6446,7 +6445,7 @@
     </c:view3D>
     <c:plotArea>
       <c:layout/>
-      <c:lineChart>
+      <c:line3DChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
@@ -6853,10 +6852,10 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:marker val="1"/>
         <c:axId val="1"/>
         <c:axId val="2"/>
-      </c:lineChart>
+        <c:gapDepth val="300"/>
+      </c:line3DChart>
       <c:catAx>
         <c:axId val="1"/>
         <c:scaling>
@@ -9999,7 +9998,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf3f9fdcb9feb462c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1fd8747d48444509"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10029,7 +10028,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rde637b8cf5794495"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R007e3221a060425a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10059,7 +10058,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R386281adf55e4bfd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b99792e48be49a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10089,7 +10088,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e1edaa5c6d14760"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf10a6b62b4a24424"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10124,7 +10123,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd8c0ee7da435434c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6755e941f12f49ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10154,7 +10153,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1463586350e94f93"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3bf6cb00e5b4b37"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10184,7 +10183,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6fdd0f1f7b864adf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7e38e17f4664949"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10214,7 +10213,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R861290005a6f4d43"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7d49f0a17b0d4998"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10249,7 +10248,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R35908d379a5f4857"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R31c30e7a8cdf4805"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10279,7 +10278,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac3bc7e1ddd94f7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R601ce7b4dc134810"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10309,7 +10308,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b31f4be218c49d7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9c0c8d6c6084516"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10339,7 +10338,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R60aed7587c18482d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfcaeada6b1df49c1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10374,7 +10373,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9fe1ec423cfe4ce8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd6e9204353744be4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10404,7 +10403,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb5f032c29a9b4cf6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2d00411f3efd4909"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10434,7 +10433,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra07bbf77f8be491e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6f5720cc581941e3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10464,7 +10463,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0f72a7bc4dbe4b23"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R861b813cd1cc4723"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10499,7 +10498,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9f33ce95f6c846bb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b29e578179c49b6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10529,7 +10528,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R11067538349f4583"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0668b0d28b3342a5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10559,7 +10558,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R755a0a0f5e914f40"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R947afb5fce0945f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10589,7 +10588,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R09bb59b08c4a49bd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfb205428431240d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10624,7 +10623,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7fcc7cb75e4a4cf6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R601242dccd104580"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10654,7 +10653,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R940cb26db4a14053"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc90a430567ef47dd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10684,7 +10683,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R826c38cf9b044615"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rffef394309804500"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10714,7 +10713,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R179dfef656c64b27"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b9aa3f427414484"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10749,7 +10748,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbcc33deba8b54711"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bf0b077149849c3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10779,7 +10778,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbac6319153cb480e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c434f2524e54303"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10809,7 +10808,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfb8fdb524c124fed"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d98715520cf450b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10839,7 +10838,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0012c76a3f634f46"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf055a04a9d846d4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -11079,48 +11078,48 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c96f304a514f1e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba62104c01a547ba"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R715f091b0bf5404a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08bdcc4aa67440b2"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38405a3b5b9f4ffe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c73af1674cf4ab5"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde387881e54548d2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b9e9a9c891403d"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca2f22405b2843d6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccfd96f4b4b34a8c"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c3e2f227e4d4f1e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0fdeb125d27413d"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3361fc1eddd4f47"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff87f1e5018a4768"/>
 </x:worksheet>
 </file>
</xml_diff>